<commit_message>
pn5180 board rev 2.0
</commit_message>
<xml_diff>
--- a/hardware/electronics/work_on_progree_pn5180_board/production/bom.xlsx
+++ b/hardware/electronics/work_on_progree_pn5180_board/production/bom.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ludwin/Elektronik/abr/hardware/electronics/pn5180_board/production/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ludwin/Elektronik/abr/hardware/electronics/work_on_progree_pn5180_board/production/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FA62D7D-EDFA-7040-9D2B-037AFDE29B81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{722BF39B-7F71-1A4A-BCCD-5C2B12B0D68E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="500" yWindow="1260" windowWidth="27840" windowHeight="16480" xr2:uid="{3A696B21-8DD3-CF4B-8C92-54C2268016F1}"/>
+    <workbookView xWindow="3760" yWindow="2300" windowWidth="27440" windowHeight="15980" xr2:uid="{F76BE561-A2DF-4147-A969-587CB2032F7F}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="bom" localSheetId="0">Tabelle1!$A$1:$E$26</definedName>
+    <definedName name="bom" localSheetId="0">Tabelle1!$A$1:$E$27</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -43,8 +43,8 @@
 
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
 <connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16">
-  <connection id="1" xr16:uid="{3AF609BB-0FD5-C241-BB3A-2AE22C60F282}" name="bom" type="6" refreshedVersion="8" background="1" saveData="1">
-    <textPr codePage="65001" sourceFile="/Users/ludwin/Elektronik/abr/hardware/electronics/pn5180_board/production/bom.csv" decimal="," thousands="." comma="1">
+  <connection id="1" xr16:uid="{27BAC9F1-2274-5E43-8791-D3AF81BBEE26}" name="bom" type="6" refreshedVersion="8" background="1" saveData="1">
+    <textPr codePage="65001" sourceFile="/Users/ludwin/Elektronik/abr/hardware/electronics/work_on_progree_pn5180_board/production/bom.csv" decimal="," thousands="." comma="1">
       <textFields count="5">
         <textField type="text"/>
         <textField type="text"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="95">
   <si>
     <t>Designator</t>
   </si>
@@ -75,12 +75,18 @@
     <t>LCSC Part #</t>
   </si>
   <si>
+    <t>C1</t>
+  </si>
+  <si>
     <t>0603</t>
   </si>
   <si>
     <t>1</t>
   </si>
   <si>
+    <t>1u</t>
+  </si>
+  <si>
     <t>C15849</t>
   </si>
   <si>
@@ -117,10 +123,10 @@
     <t>2</t>
   </si>
   <si>
-    <t>1.5 pF</t>
-  </si>
-  <si>
-    <t>C1552</t>
+    <t>1nF</t>
+  </si>
+  <si>
+    <t>C1523</t>
   </si>
   <si>
     <t>C16, C20</t>
@@ -132,55 +138,55 @@
     <t>C1548</t>
   </si>
   <si>
-    <t>C17, C18, C33, C34</t>
+    <t>C17, C18</t>
+  </si>
+  <si>
+    <t>56pF</t>
+  </si>
+  <si>
+    <t>C39148</t>
+  </si>
+  <si>
+    <t>C19</t>
+  </si>
+  <si>
+    <t>10uF</t>
+  </si>
+  <si>
+    <t>C96446</t>
+  </si>
+  <si>
+    <t>C21, C22, C35, C36</t>
   </si>
   <si>
     <t>4</t>
   </si>
   <si>
+    <t>68pF</t>
+  </si>
+  <si>
+    <t>C28262</t>
+  </si>
+  <si>
+    <t>C29, C30</t>
+  </si>
+  <si>
+    <t>47pF</t>
+  </si>
+  <si>
+    <t>C1671</t>
+  </si>
+  <si>
+    <t>C33, C34</t>
+  </si>
+  <si>
     <t>100pF</t>
   </si>
   <si>
     <t>C14858</t>
   </si>
   <si>
-    <t>C19</t>
-  </si>
-  <si>
-    <t>10uF</t>
-  </si>
-  <si>
-    <t>C96446</t>
-  </si>
-  <si>
-    <t>C21, C22</t>
-  </si>
-  <si>
-    <t>27pF</t>
-  </si>
-  <si>
-    <t>C28, C31</t>
-  </si>
-  <si>
-    <t>C1644</t>
-  </si>
-  <si>
-    <t>C29, C30</t>
-  </si>
-  <si>
-    <t>68pF</t>
-  </si>
-  <si>
-    <t>C28262</t>
-  </si>
-  <si>
-    <t>C35, C36</t>
-  </si>
-  <si>
-    <t>22pF</t>
-  </si>
-  <si>
-    <t>C1653</t>
+    <t>C37</t>
   </si>
   <si>
     <t>1µF</t>
@@ -240,10 +246,10 @@
     <t>R10, R11</t>
   </si>
   <si>
-    <t>2R7</t>
-  </si>
-  <si>
-    <t>C2930033</t>
+    <t>2Ohm</t>
+  </si>
+  <si>
+    <t>C22977</t>
   </si>
   <si>
     <t>R13, R8</t>
@@ -255,6 +261,15 @@
     <t>C25741</t>
   </si>
   <si>
+    <t>R14, R17</t>
+  </si>
+  <si>
+    <t>1Ohm</t>
+  </si>
+  <si>
+    <t>C22936</t>
+  </si>
+  <si>
     <t>R2, R3</t>
   </si>
   <si>
@@ -328,12 +343,6 @@
   </si>
   <si>
     <t>C29975</t>
-  </si>
-  <si>
-    <t>C1, C37</t>
-  </si>
-  <si>
-    <t>C107045</t>
   </si>
 </sst>
 </file>
@@ -390,7 +399,7 @@
 </file>
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="bom" connectionId="1" xr16:uid="{1ABF5E6B-B889-0D40-AA9F-5A82077341F4}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="bom" connectionId="1" xr16:uid="{0F657D60-0E0A-BC4B-8B89-3FA2D6270F3E}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -709,8 +718,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B868FD3B-987E-7B43-8526-D9BF79C23C73}">
-  <dimension ref="A1:E26"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{129C5684-192B-8F47-AA1E-7C755011E4C2}">
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.1640625" bestFit="1" customWidth="1"/>
@@ -739,427 +748,444 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>18</v>
-      </c>
       <c r="D9" s="1" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>90</v>
+        <v>42</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>75</v>
+        <v>11</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>